<commit_message>
Fix winner time: use last competitive round, not solo cup-end round
The Eggy cup-end winner-marker round (only the winner left, then 'eliminated'
by the mod as an end signal) logs a meaningless time, often DNF since the
winner doesn't finish a solo lap. new_cup.py was grabbing that as the winner's
displayed time. Now it skips the solo marker round and uses the last round the
winner actually raced someone. Eggy 93 winner justMaki: DNF -> 25.347.
</commit_message>
<xml_diff>
--- a/Eggy Cup 87-93.xlsx
+++ b/Eggy Cup 87-93.xlsx
@@ -745,10 +745,8 @@
           <t>justMaki</t>
         </is>
       </c>
-      <c r="AM6" t="inlineStr">
-        <is>
-          <t>DNF</t>
-        </is>
+      <c r="AM6" t="n">
+        <v>25347</v>
       </c>
     </row>
     <row r="7">

</xml_diff>